<commit_message>
Daily slate 2026-06-13 [auto]
</commit_message>
<xml_diff>
--- a/ui_runner/templates/graded_analysis_tabs_2026-06-12.xlsx
+++ b/ui_runner/templates/graded_analysis_tabs_2026-06-12.xlsx
@@ -471,16 +471,16 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>39</v>
+        <v>67</v>
       </c>
       <c r="E2" t="n">
-        <v>16</v>
+        <v>35</v>
       </c>
       <c r="F2" t="n">
-        <v>23</v>
+        <v>32</v>
       </c>
       <c r="G2" t="n">
-        <v>41</v>
+        <v>52.2</v>
       </c>
     </row>
     <row r="3">
@@ -500,16 +500,16 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>203</v>
+        <v>247</v>
       </c>
       <c r="E3" t="n">
-        <v>106</v>
+        <v>131</v>
       </c>
       <c r="F3" t="n">
-        <v>97</v>
+        <v>116</v>
       </c>
       <c r="G3" t="n">
-        <v>52.2</v>
+        <v>53</v>
       </c>
     </row>
     <row r="4">
@@ -558,13 +558,16 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="E5" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F5" t="n">
-        <v>0</v>
+        <v>3</v>
+      </c>
+      <c r="G5" t="n">
+        <v>50</v>
       </c>
     </row>
     <row r="6">
@@ -636,16 +639,16 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>55</v>
+        <v>81</v>
       </c>
       <c r="E8" t="n">
-        <v>18</v>
+        <v>32</v>
       </c>
       <c r="F8" t="n">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="G8" t="n">
-        <v>32.7</v>
+        <v>39.5</v>
       </c>
     </row>
     <row r="9">
@@ -665,16 +668,16 @@
         </is>
       </c>
       <c r="D9" t="n">
+        <v>9</v>
+      </c>
+      <c r="E9" t="n">
+        <v>8</v>
+      </c>
+      <c r="F9" t="n">
         <v>1</v>
       </c>
-      <c r="E9" t="n">
-        <v>1</v>
-      </c>
-      <c r="F9" t="n">
-        <v>0</v>
-      </c>
       <c r="G9" t="n">
-        <v>100</v>
+        <v>88.90000000000001</v>
       </c>
     </row>
     <row r="10">
@@ -694,16 +697,16 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>96</v>
+        <v>132</v>
       </c>
       <c r="E10" t="n">
-        <v>56</v>
+        <v>78</v>
       </c>
       <c r="F10" t="n">
-        <v>40</v>
+        <v>54</v>
       </c>
       <c r="G10" t="n">
-        <v>58.3</v>
+        <v>59.1</v>
       </c>
     </row>
     <row r="11">
@@ -723,16 +726,16 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>1052</v>
+        <v>1082</v>
       </c>
       <c r="E11" t="n">
-        <v>633</v>
+        <v>647</v>
       </c>
       <c r="F11" t="n">
-        <v>419</v>
+        <v>435</v>
       </c>
       <c r="G11" t="n">
-        <v>60.2</v>
+        <v>59.8</v>
       </c>
     </row>
     <row r="12">
@@ -752,16 +755,16 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>140</v>
+        <v>150</v>
       </c>
       <c r="E12" t="n">
-        <v>93</v>
+        <v>100</v>
       </c>
       <c r="F12" t="n">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="G12" t="n">
-        <v>66.40000000000001</v>
+        <v>66.7</v>
       </c>
     </row>
     <row r="13">
@@ -781,16 +784,16 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>84</v>
+        <v>94</v>
       </c>
       <c r="E13" t="n">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="F13" t="n">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="G13" t="n">
-        <v>35.7</v>
+        <v>39.4</v>
       </c>
     </row>
     <row r="14">
@@ -810,16 +813,16 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>275</v>
+        <v>284</v>
       </c>
       <c r="E14" t="n">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="F14" t="n">
-        <v>202</v>
+        <v>208</v>
       </c>
       <c r="G14" t="n">
-        <v>26.5</v>
+        <v>26.8</v>
       </c>
     </row>
     <row r="15">
@@ -839,16 +842,16 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>323</v>
+        <v>364</v>
       </c>
       <c r="E15" t="n">
-        <v>68</v>
+        <v>81</v>
       </c>
       <c r="F15" t="n">
-        <v>255</v>
+        <v>283</v>
       </c>
       <c r="G15" t="n">
-        <v>21.1</v>
+        <v>22.3</v>
       </c>
     </row>
     <row r="16">
@@ -868,16 +871,16 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>107</v>
+        <v>161</v>
       </c>
       <c r="E16" t="n">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="F16" t="n">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="G16" t="n">
-        <v>15</v>
+        <v>19.9</v>
       </c>
     </row>
     <row r="17">
@@ -897,13 +900,13 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>4307</v>
+        <v>4371</v>
       </c>
       <c r="E17" t="n">
-        <v>914</v>
+        <v>925</v>
       </c>
       <c r="F17" t="n">
-        <v>3393</v>
+        <v>3446</v>
       </c>
       <c r="G17" t="n">
         <v>21.2</v>
@@ -1096,32 +1099,59 @@
           <t>Elite</t>
         </is>
       </c>
+      <c r="B2" t="n">
+        <v>61.1</v>
+      </c>
       <c r="C2" t="n">
-        <v>0</v>
+        <v>36</v>
+      </c>
+      <c r="D2" t="n">
+        <v>46.7</v>
       </c>
       <c r="E2" t="n">
-        <v>0</v>
+        <v>30</v>
+      </c>
+      <c r="F2" t="n">
+        <v>70</v>
       </c>
       <c r="G2" t="n">
-        <v>0</v>
+        <v>10</v>
+      </c>
+      <c r="H2" t="n">
+        <v>70</v>
       </c>
       <c r="I2" t="n">
-        <v>0</v>
+        <v>10</v>
+      </c>
+      <c r="J2" t="n">
+        <v>33.3</v>
       </c>
       <c r="K2" t="n">
-        <v>0</v>
+        <v>9</v>
+      </c>
+      <c r="L2" t="n">
+        <v>31.7</v>
       </c>
       <c r="M2" t="n">
-        <v>0</v>
+        <v>41</v>
+      </c>
+      <c r="N2" t="n">
+        <v>29.6</v>
       </c>
       <c r="O2" t="n">
-        <v>0</v>
+        <v>54</v>
+      </c>
+      <c r="P2" t="n">
+        <v>17.2</v>
       </c>
       <c r="Q2" t="n">
-        <v>0</v>
+        <v>64</v>
+      </c>
+      <c r="R2" t="n">
+        <v>70.40000000000001</v>
       </c>
       <c r="S2" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="U2" t="n">
         <v>0</v>
@@ -1129,20 +1159,32 @@
       <c r="W2" t="n">
         <v>0</v>
       </c>
+      <c r="X2" t="n">
+        <v>50</v>
+      </c>
       <c r="Y2" t="n">
-        <v>0</v>
+        <v>22</v>
+      </c>
+      <c r="Z2" t="n">
+        <v>59.5</v>
       </c>
       <c r="AA2" t="n">
-        <v>0</v>
+        <v>37</v>
+      </c>
+      <c r="AB2" t="n">
+        <v>50</v>
       </c>
       <c r="AC2" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AE2" t="n">
         <v>0</v>
       </c>
+      <c r="AF2" t="n">
+        <v>87.5</v>
+      </c>
       <c r="AG2" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
     </row>
     <row r="3">
@@ -1441,58 +1483,58 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>58.3</v>
+        <v>59.1</v>
       </c>
       <c r="C7" t="n">
-        <v>96</v>
+        <v>132</v>
       </c>
       <c r="D7" t="n">
-        <v>60.2</v>
+        <v>59.8</v>
       </c>
       <c r="E7" t="n">
-        <v>1052</v>
+        <v>1082</v>
       </c>
       <c r="F7" t="n">
-        <v>66.40000000000001</v>
+        <v>66.7</v>
       </c>
       <c r="G7" t="n">
-        <v>140</v>
+        <v>150</v>
       </c>
       <c r="H7" t="n">
-        <v>35.7</v>
+        <v>39.4</v>
       </c>
       <c r="I7" t="n">
-        <v>84</v>
+        <v>94</v>
       </c>
       <c r="J7" t="n">
-        <v>26.5</v>
+        <v>26.8</v>
       </c>
       <c r="K7" t="n">
-        <v>275</v>
+        <v>284</v>
       </c>
       <c r="L7" t="n">
-        <v>21.1</v>
+        <v>22.3</v>
       </c>
       <c r="M7" t="n">
-        <v>323</v>
+        <v>364</v>
       </c>
       <c r="N7" t="n">
-        <v>15</v>
+        <v>19.9</v>
       </c>
       <c r="O7" t="n">
-        <v>107</v>
+        <v>161</v>
       </c>
       <c r="P7" t="n">
         <v>21.2</v>
       </c>
       <c r="Q7" t="n">
-        <v>4307</v>
+        <v>4371</v>
       </c>
       <c r="R7" t="n">
-        <v>41</v>
+        <v>52.2</v>
       </c>
       <c r="S7" t="n">
-        <v>39</v>
+        <v>67</v>
       </c>
       <c r="T7" t="n">
         <v>46.4</v>
@@ -1504,28 +1546,31 @@
         <v>0</v>
       </c>
       <c r="X7" t="n">
-        <v>32.7</v>
+        <v>39.5</v>
       </c>
       <c r="Y7" t="n">
-        <v>55</v>
+        <v>81</v>
       </c>
       <c r="Z7" t="n">
-        <v>52.2</v>
+        <v>53</v>
       </c>
       <c r="AA7" t="n">
-        <v>203</v>
+        <v>247</v>
+      </c>
+      <c r="AB7" t="n">
+        <v>50</v>
       </c>
       <c r="AC7" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AE7" t="n">
         <v>0</v>
       </c>
       <c r="AF7" t="n">
-        <v>100</v>
+        <v>88.90000000000001</v>
       </c>
       <c r="AG7" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>